<commit_message>
Record that the ED pools and E/M are four separate populations
The same encounter coded for the facility, coded professionally and coded
single-path is three different charts, and none of them belongs in the E/M
pool. Two of the workbook's open decisions turned on this, so both are now
settled rather than outstanding.

What it changes: the four pools add rather than overlap, so nothing is
double-counted and the ED requirement is not overstated. The cost lands on
sourcing instead -- four distinct pulls, not one pull classified four ways --
and the E/M topic list holding no ED setting is deliberate.

The Decisions sheet gains a status column so a settled decision carries what
was decided rather than disappearing from the record.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GAgNTxNNybv6W7GXL33G6z
</commit_message>
<xml_diff>
--- a/docs/PracticeLab_Chart_Composition_Taxonomy.xlsx
+++ b/docs/PracticeLab_Chart_Composition_Taxonomy.xlsx
@@ -30,7 +30,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,6 +73,16 @@
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002E7D32"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B23A33"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="8">
@@ -139,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -224,6 +234,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -591,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -759,50 +781,72 @@
     <row r="22">
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>What the targets are and are not</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="39" customHeight="1">
+          <t>The four populations are separate</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="52" customHeight="1">
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>A target is a proportion of a pool, not a forecast of what production will yield. Where the two disagree the pool is wrong, not the sheet: a pool that drifts toward whatever charts were easy to find teaches whatever those charts happened to contain.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="26" customHeight="1">
+          <t>ED Facility, ED Profee, ED Single Path and E/M are four distinct chart populations, confirmed on 15 October 2026. The same clinical encounter coded for the facility, coded professionally, and coded single-path produces three different charts, and none of them sits in the E/M pool. Their pools therefore add rather than overlap, and the E/M topic list holding no ED setting is deliberate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="52" customHeight="1">
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Rounding is per topic, so the sum of targets can differ from the pool by a chart or two. Each sheet shows the variance rather than hiding it, and the pool is the authority.</t>
+          <t>The consequence for sourcing is the part worth saying out loud: four populations means four separate pulls, not one pull classified four ways. A chart cannot be filed under an ED Facility topic and an ED Profee topic at once, and reusing one encounter across two pools would put the same documentation in front of a coder twice under two different names.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Scope</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="52" customHeight="1">
+          <t>What the targets are and are not</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="39" customHeight="1">
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Seven specialties. IP-DRG, ED Facility, E/M and SDS carry HC baseline pools. ED Profee, Surgery and ED Single Path each carry a pool set on 15 October 2026 (400, 300 and 300) rather than one derived in the HC model. Denials/Edits and Ancillary are deferred — their HC pools and coverage matrices stand, and a topic layer for them is the obvious next addition.</t>
+          <t>A target is a proportion of a pool, not a forecast of what production will yield. Where the two disagree the pool is wrong, not the sheet: a pool that drifts toward whatever charts were easy to find teaches whatever those charts happened to contain.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="26" customHeight="1">
       <c r="B28" s="4" t="inlineStr">
         <is>
+          <t>Rounding is per topic, so the sum of targets can differ from the pool by a chart or two. Each sheet shows the variance rather than hiding it, and the pool is the authority.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="52" customHeight="1">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Seven specialties. IP-DRG, ED Facility, E/M and SDS carry HC baseline pools. ED Profee, Surgery and ED Single Path each carry a pool set on 15 October 2026 (400, 300 and 300) rather than one derived in the HC model. Denials/Edits and Ancillary are deferred — their HC pools and coverage matrices stand, and a topic layer for them is the obvious next addition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
+      <c r="B32" s="4" t="inlineStr">
+        <is>
           <t>Open questions that need a decision before this is final are on the Open Decisions sheet. They are listed rather than resolved because each changes a number somebody else owns.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="16">
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="B5:C5"/>
@@ -810,6 +854,8 @@
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B31:C31"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="A2:C2"/>
@@ -824,7 +870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1746,26 +1792,34 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="26" customHeight="1">
+    <row r="46" ht="39" customHeight="1">
       <c r="A46" s="15" t="inlineStr">
         <is>
-          <t>Severity on IP-DRG and Method on E/M are cross-cutting dimensions: a chart has a CC/MCC status and an MDM-or-time basis whatever its topic. They are checked across the pool, not decomposed per topic, which is why the topic sheets carry one dimension each.</t>
+          <t>ED Facility, ED Profee and ED Single Path are three separate populations, not three views of one. The same encounter coded for the facility, coded professionally and coded single-path is three different charts; none of them belongs in the E/M pool, which is why the E/M dimension here has no ED setting. Confirmed 15 October 2026.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="26" customHeight="1">
       <c r="A47" s="15" t="inlineStr">
         <is>
+          <t>Severity on IP-DRG and Method on E/M are cross-cutting dimensions: a chart has a CC/MCC status and an MDM-or-time basis whatever its topic. They are checked across the pool, not decomposed per topic, which is why the topic sheets carry one dimension each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="26" customHeight="1">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
           <t>Where a target percentage here changes, the matching band row on the topic sheet and its child weights must change together. The band row's check cell is what tells you they have come apart.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A47:F47"/>
+    <mergeCell ref="A46:F46"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A48:F48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2087,26 +2141,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="72" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Open decisions</t>
+          <t>Decisions</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Each one changes a number somebody else owns, so they are listed rather than resolved. Nothing on the topic sheets depends on them being settled first.</t>
+          <t>Settled ones first, with what was decided. The open ones each change a number somebody else owns, so they are listed rather than resolved — nothing on the topic sheets depends on them being settled first.</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2178,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>What is at stake</t>
+          <t>What is at stake, or what was decided</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -2131,64 +2186,84 @@
           <t>Owner</t>
         </is>
       </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="66" customHeight="1">
-      <c r="A5" s="24" t="n">
+      <c r="A5" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="21" t="inlineStr">
-        <is>
-          <t>Add ED Profee, Surgery and ED Single Path to the HC model</t>
-        </is>
-      </c>
-      <c r="C5" s="22" t="inlineStr">
-        <is>
-          <t>Pools of 400, 300 and 300 were set here, outside the HC model. None of them has a +10% buffer calculation, a per-batch average, a batch count or a build-hour line. That is 1,000 charts the HC Specialty Grid, Chart Pool, FTE Demand and FTE Summary sheets do not know about — at HC's own build rates roughly 1,500 to 2,250 hours, close to a further FTE. Until they are added, the team size in that model is understated.</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>Whoever owns the HC model</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="55" customHeight="1">
-      <c r="A6" s="24" t="n">
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>ED Facility, ED Profee, ED Single Path and E/M are four separate chart populations</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>Confirmed: an ED encounter coded for the facility, the same encounter coded professionally, and a single-path encounter are three different charts, and none of them belongs in the E/M pool. So the pools of 704, 400, 300 and 413 do not overlap and nothing is double-counted — but sourcing has to pull four distinct populations, and the E/M pool holding no ED setting is correct rather than an oversight.</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="inlineStr">
+        <is>
+          <t>Confirmed by the user</t>
+        </is>
+      </c>
+      <c r="E5" s="36" t="inlineStr">
+        <is>
+          <t>Settled 2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>Confirm ED Profee and ED Single Path do not double-count ED Facility</t>
-        </is>
-      </c>
-      <c r="C6" s="22" t="inlineStr">
-        <is>
-          <t>One ED encounter can be coded facility-only, profee-only or single-path. Three pools of 704, 400 and 300 assume three distinct chart populations. If the same encounters are being counted twice, the ED requirement is overstated by up to 700 charts; if they genuinely are distinct, sourcing has to pull three times from the same production stream.</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>PL Trainer, ED specialties</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>E/M keeps no ED-setting share</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>Follows from the above. ED E/M sits in ED Profee, the E/M topic list deliberately holds no ED setting, and the HC E/M pool of 413 is not oversized by it.</t>
+        </is>
+      </c>
+      <c r="D6" s="32" t="inlineStr">
+        <is>
+          <t>Confirmed by the user</t>
+        </is>
+      </c>
+      <c r="E6" s="36" t="inlineStr">
+        <is>
+          <t>Settled 2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="77" customHeight="1">
       <c r="A7" s="24" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="21" t="inlineStr">
         <is>
-          <t>Decide whether E/M keeps an ED-setting share</t>
+          <t>Add ED Profee, Surgery and ED Single Path to the HC model</t>
         </is>
       </c>
       <c r="C7" s="22" t="inlineStr">
         <is>
-          <t>ED E/M now sits in ED Profee, so the E/M topic list deliberately holds no ED setting. If the HC E/M pool of 413 was sized including ED visits, it is now oversized by that share and the ED Profee 400 partly duplicates it.</t>
+          <t>Pools of 400, 300 and 300 were set here, outside the HC model. None of them has a +10% buffer calculation, a per-batch average, a batch count or a build-hour line. That is 1,000 charts the HC Specialty Grid, Chart Pool, FTE Demand and FTE Summary sheets do not know about — at HC's own build rates roughly 1,500 to 2,250 hours, close to a further FTE. Until they are added, the team size in that model is understated.</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>PL Trainer, E/M</t>
+          <t>Whoever owns the HC model</t>
+        </is>
+      </c>
+      <c r="E7" s="37" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2211,8 +2286,13 @@
           <t>PL Trainer plus QR</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="44" customHeight="1">
+      <c r="E8" s="37" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="55" customHeight="1">
       <c r="A9" s="24" t="n">
         <v>5</v>
       </c>
@@ -2231,8 +2311,13 @@
           <t>PL Trainer plus Compliance for X2</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
+      <c r="E9" s="37" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
       <c r="A10" s="24" t="n">
         <v>6</v>
       </c>
@@ -2251,8 +2336,13 @@
           <t>PL Trainer plus the platform team</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
+      <c r="E10" s="37" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1">
       <c r="A11" s="24" t="n">
         <v>7</v>
       </c>
@@ -2269,6 +2359,11 @@
       <c r="D11" s="11" t="inlineStr">
         <is>
           <t>PL Trainer</t>
+        </is>
+      </c>
+      <c r="E11" s="37" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2291,11 +2386,16 @@
           <t>PL Trainer, at the first refresh</t>
         </is>
       </c>
+      <c r="E12" s="37" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>